<commit_message>
feat(ci): add AST registry extractor, validator guard F-058, and probe hooks
- Implement scripts/extract_registries.py for AST-based registry discovery, component extraction, and doc drift detection.
- Add scripts/validations/F_058.py 5-point sweep guard ensuring features.yaml, validation scripts, test modules, and CI coverage configs remain in sync.
- Consolidate subprocess probe logic into tests/registry_probe_hook.py and tests/_registry_probe.py.
- Standardize entrypoints across all F_*.py validation modules with canonical main() callables.
- Add tests/test_extract_registries.py with 20 unit, integration, and CLI tests.
- Update .github/workflows/docs.yml and quality-gates.yml to invoke the new tools and enforce coverage.
- Sync CHANGELOG.md, NEXT_STEPS.md, and README.md.
</commit_message>
<xml_diff>
--- a/docs/e2e-matrix/e2e-test-matrix.xlsx
+++ b/docs/e2e-matrix/e2e-test-matrix.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Test Matrix" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Coverage Grid" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Credentials" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Provenance" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage Grid" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Credentials" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Provenance" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Matrix'!$A$1:$N$41</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Summary'!$A$1:$B$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Summary'!$A$1:$B$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Coverage Grid'!$A$1:$G$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Credentials'!$A$1:$C$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Provenance'!$A$1:$B$9</definedName>
@@ -40,7 +40,7 @@
       <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -62,11 +62,6 @@
         <fgColor rgb="FFE6E6E6"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFBEFCB"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -80,12 +75,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -576,17 +570,17 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>790 tests</t>
+          <t>714 tests</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>81447</t>
+          <t>47591</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>790</t>
+          <t>714</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -644,17 +638,17 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>157 tests</t>
+          <t>89 tests</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>47263</t>
+          <t>20250</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>157</t>
+          <t>89</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -717,7 +711,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>7135</t>
+          <t>6791</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -737,7 +731,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -780,17 +774,17 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>163 tests</t>
+          <t>119 tests</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>14537</t>
+          <t>4876</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>163</t>
+          <t>119</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -853,7 +847,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>3921</t>
+          <t>2389</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -916,17 +910,17 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1627 tests</t>
+          <t>995 tests</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>85040</t>
+          <t>40601</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>1627</t>
+          <t>995</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -941,7 +935,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>11</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -984,17 +978,17 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1627 tests</t>
+          <t>995 tests</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>61257</t>
+          <t>39940</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>1627</t>
+          <t>995</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1009,7 +1003,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>11</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1053,7 +1047,7 @@
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>44902</t>
+          <t>33088</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
@@ -1093,26 +1087,22 @@
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>1590</t>
-        </is>
-      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>NOT-RUN</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>not reached in this run</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>artifacts/e2e-report/matrix_coverage-check.log</t>
-        </is>
-      </c>
+      <c r="N10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1149,7 +1139,7 @@
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>644</t>
+          <t>516</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
@@ -1197,7 +1187,7 @@
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>585</t>
+          <t>506</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
@@ -1245,7 +1235,7 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>643</t>
+          <t>531</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
@@ -1293,7 +1283,7 @@
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>1687</t>
+          <t>1166</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
@@ -1381,7 +1371,7 @@
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>621</t>
+          <t>595</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
@@ -1429,7 +1419,7 @@
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>599</t>
+          <t>520</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
@@ -1477,7 +1467,7 @@
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>1186</t>
+          <t>1094</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
@@ -1525,7 +1515,7 @@
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>1222</t>
+          <t>1045</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
@@ -1573,7 +1563,7 @@
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>1247</t>
+          <t>1114</t>
         </is>
       </c>
       <c r="J20" t="inlineStr"/>
@@ -1621,7 +1611,7 @@
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>1208</t>
+          <t>1173</t>
         </is>
       </c>
       <c r="J21" t="inlineStr"/>
@@ -1669,7 +1659,7 @@
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>1108</t>
+          <t>1144</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
@@ -1717,7 +1707,7 @@
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>1160</t>
+          <t>1098</t>
         </is>
       </c>
       <c r="J23" t="inlineStr"/>
@@ -1769,7 +1759,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>651</t>
+          <t>534</t>
         </is>
       </c>
       <c r="J24" t="inlineStr"/>
@@ -1817,7 +1807,7 @@
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>660</t>
+          <t>595</t>
         </is>
       </c>
       <c r="J25" t="inlineStr"/>
@@ -1865,7 +1855,7 @@
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
-          <t>582</t>
+          <t>571</t>
         </is>
       </c>
       <c r="J26" t="inlineStr"/>
@@ -1913,7 +1903,7 @@
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>602</t>
+          <t>512</t>
         </is>
       </c>
       <c r="J27" t="inlineStr"/>
@@ -2001,7 +1991,7 @@
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>568</t>
+          <t>456</t>
         </is>
       </c>
       <c r="J29" t="inlineStr"/>
@@ -2049,7 +2039,7 @@
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
-          <t>732</t>
+          <t>605</t>
         </is>
       </c>
       <c r="J30" t="inlineStr"/>
@@ -2101,7 +2091,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>17666</t>
+          <t>16544</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -2169,7 +2159,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>12607</t>
+          <t>7594</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -2189,7 +2179,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -2229,21 +2219,17 @@
           <t>ANTHROPIC_API_KEY</t>
         </is>
       </c>
-      <c r="G33" s="4" t="inlineStr">
-        <is>
-          <t>SKIP</t>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>NOT-RUN</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>ANTHROPIC_API_KEY not set</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>not reached in this run</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr"/>
@@ -2281,21 +2267,17 @@
           <t>AWS_ACCESS_KEY_ID, AWS_SECRET_ACCESS_KEY</t>
         </is>
       </c>
-      <c r="G34" s="4" t="inlineStr">
-        <is>
-          <t>SKIP</t>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>NOT-RUN</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>AWS_ACCESS_KEY_ID,AWS_SECRET_ACCESS_KEY not set</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>not reached in this run</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr"/>
@@ -2333,21 +2315,17 @@
           <t>OPENAI_API_KEY</t>
         </is>
       </c>
-      <c r="G35" s="4" t="inlineStr">
-        <is>
-          <t>SKIP</t>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>NOT-RUN</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>OPENAI_API_KEY not set</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>not reached in this run</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr"/>
@@ -2385,21 +2363,17 @@
           <t>LANGFUSE_SECRET_KEY, LANGFUSE_PUBLIC_KEY, LANGFUSE_BASE_URL</t>
         </is>
       </c>
-      <c r="G36" s="4" t="inlineStr">
-        <is>
-          <t>SKIP</t>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>NOT-RUN</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>LANGFUSE_* not set</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>not reached in this run</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr"/>
@@ -2437,21 +2411,17 @@
           <t>LANGFUSE_SECRET_KEY, LANGFUSE_PUBLIC_KEY, LANGFUSE_BASE_URL</t>
         </is>
       </c>
-      <c r="G37" s="4" t="inlineStr">
-        <is>
-          <t>SKIP</t>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>NOT-RUN</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>LANGFUSE_* not set</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>not reached in this run</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr"/>
@@ -2489,21 +2459,17 @@
           <t>PHOENIX_COLLECTOR_ENDPOINT</t>
         </is>
       </c>
-      <c r="G38" s="4" t="inlineStr">
-        <is>
-          <t>SKIP</t>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>NOT-RUN</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>PHOENIX_COLLECTOR_ENDPOINT not set</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>not reached in this run</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr"/>
@@ -2541,21 +2507,17 @@
           <t>PHOENIX_COLLECTOR_ENDPOINT</t>
         </is>
       </c>
-      <c r="G39" s="4" t="inlineStr">
-        <is>
-          <t>SKIP</t>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>NOT-RUN</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>PHOENIX_COLLECTOR_ENDPOINT not set</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>not reached in this run</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr"/>
@@ -2666,7 +2628,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2705,7 +2667,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>30</t>
         </is>
       </c>
     </row>
@@ -2717,7 +2679,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>10</t>
         </is>
       </c>
     </row>
@@ -2729,96 +2691,84 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>30</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Status SKIP</t>
+          <t>Tier A</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>PASS 7</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Tier A</t>
+          <t>Tier B</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>PASS 7</t>
+          <t>PASS 1</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Tier B</t>
+          <t>Tier C</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>PASS 2</t>
+          <t>PASS 21</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Tier C</t>
+          <t>Tier D</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>PASS 21</t>
+          <t>not exercised in this run</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Tier D</t>
+          <t>Tier E</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>SKIP 7</t>
+          <t>not exercised in this run</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Tier E</t>
+          <t>Tier PRE</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>not exercised in this run</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Tier PRE</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
           <t>PASS 1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B12"/>
+  <autoFilter ref="A1:B11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2911,7 +2861,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>790</t>
+          <t>714</t>
         </is>
       </c>
     </row>
@@ -2948,7 +2898,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>157</t>
+          <t>89</t>
         </is>
       </c>
     </row>
@@ -3055,7 +3005,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>163</t>
+          <t>119</t>
         </is>
       </c>
     </row>
@@ -3114,7 +3064,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>architecture-drift.yml, docs.yml, eval-harness-ci.yml, merge-gate-audit.yml, merge-gate-seed.yml, merge-gate-verdict.yml, outcome-labeller.yml, phoenix-live.yml, quality-gates.yml</t>
+          <t>architecture-drift.yml, docs.yml, eval-harness-ci.yml, merge-gate-audit.yml, merge-gate-seed.yml, merge-gate-verdict.yml, nightly-e2e.yml, outcome-labeller.yml, phoenix-live.yml, quality-gates.yml</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -3129,7 +3079,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>1627</t>
+          <t>995</t>
         </is>
       </c>
     </row>
@@ -3162,7 +3112,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>1627</t>
+          <t>995</t>
         </is>
       </c>
     </row>
@@ -3216,7 +3166,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SKIP</t>
+          <t>NOT-RUN</t>
         </is>
       </c>
     </row>
@@ -3233,7 +3183,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>SKIP</t>
+          <t>NOT-RUN</t>
         </is>
       </c>
     </row>
@@ -3250,7 +3200,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>SKIP</t>
+          <t>NOT-RUN</t>
         </is>
       </c>
     </row>
@@ -3267,7 +3217,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>SKIP</t>
+          <t>NOT-RUN</t>
         </is>
       </c>
     </row>
@@ -3284,7 +3234,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>SKIP</t>
+          <t>NOT-RUN</t>
         </is>
       </c>
     </row>
@@ -3301,7 +3251,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>SKIP</t>
+          <t>NOT-RUN</t>
         </is>
       </c>
     </row>
@@ -3318,7 +3268,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>SKIP</t>
+          <t>NOT-RUN</t>
         </is>
       </c>
     </row>
@@ -3361,7 +3311,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>e899249a070b1537bfd714669bc2b0adaef0573a</t>
+          <t>09337aec16e8b10588efd0e61c9d270d18ada1c4</t>
         </is>
       </c>
     </row>
@@ -3373,7 +3323,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>claude/e2e-test-plan-matrix-u6c1en</t>
+          <t>main</t>
         </is>
       </c>
     </row>
@@ -3385,7 +3335,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-08-13T21:45:54+00:00</t>
+          <t>2026-08-19T03:28:29+00:00</t>
         </is>
       </c>
     </row>
@@ -3397,7 +3347,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Linux-6.18.5-fc-v20-x86_64-with-glibc2.39</t>
+          <t>Windows-10-10.0.26200-SP0</t>
         </is>
       </c>
     </row>
@@ -3409,7 +3359,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>3.11.15</t>
+          <t>3.11.9</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(ci): POSIX e2e driver and CI-restored e2e-matrix freshness
scripts/run_all_e2e.sh mirrors the PowerShell driver (same tiers, step
inventory, report layout, anti-vacuous guards) so the nightly workflow
can produce a run report on ubuntu-latest; tests/test_e2e_driver_parity.py
fails if the two drivers drift. Freshness becomes CI-runnable via two
fixes: the Duration (ms) column is masked in the comparison (wall-clock
values can never reproduce across machines), and the committed artifact
is regenerated from the canonical Linux environment. nightly-e2e.yml
gains a single-version e2e-freshness job running driver + --check.

Co-authored-by: Ian Cruickshank <ianshank@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/e2e-matrix/e2e-test-matrix.xlsx
+++ b/docs/e2e-matrix/e2e-test-matrix.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage Grid" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Credentials" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Provenance" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Test Matrix" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Coverage Grid" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Credentials" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Provenance" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Matrix'!$A$1:$N$41</definedName>
@@ -570,17 +570,17 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>714 tests</t>
+          <t>921 tests</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>47591</t>
+          <t>10000</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>714</t>
+          <t>921</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -638,17 +638,17 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>89 tests</t>
+          <t>161 tests</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>20250</t>
+          <t>23000</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>89</t>
+          <t>161</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -706,17 +706,17 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>136 tests</t>
+          <t>140 tests</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>6791</t>
+          <t>2000</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>136</t>
+          <t>140</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -774,17 +774,17 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>119 tests</t>
+          <t>163 tests</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>4876</t>
+          <t>2000</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>119</t>
+          <t>163</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2389</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -910,22 +910,22 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>995 tests</t>
+          <t>2571 tests</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>40601</t>
+          <t>56000</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>995</t>
+          <t>2571</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>28</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -978,22 +978,22 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>995 tests</t>
+          <t>2571 tests</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>39940</t>
+          <t>55000</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>995</t>
+          <t>2571</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>28</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1047,7 +1047,7 @@
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>33088</t>
+          <t>20000</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
@@ -1087,22 +1087,26 @@
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>NOT-RUN</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>not reached in this run</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>artifacts/e2e-report/matrix_coverage-check.log</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1139,7 +1143,7 @@
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>516</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
@@ -1187,7 +1191,7 @@
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>506</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
@@ -1235,7 +1239,7 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>531</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
@@ -1283,7 +1287,7 @@
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>1166</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
@@ -1371,7 +1375,7 @@
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>595</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
@@ -1419,7 +1423,7 @@
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
@@ -1467,7 +1471,7 @@
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>1094</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
@@ -1515,7 +1519,7 @@
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>1045</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
@@ -1563,7 +1567,7 @@
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>1114</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="J20" t="inlineStr"/>
@@ -1611,7 +1615,7 @@
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>1173</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J21" t="inlineStr"/>
@@ -1659,7 +1663,7 @@
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>1144</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
@@ -1707,7 +1711,7 @@
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>1098</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J23" t="inlineStr"/>
@@ -1754,12 +1758,12 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>decision exit 10</t>
+          <t>decision</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>534</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J24" t="inlineStr"/>
@@ -1807,7 +1811,7 @@
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>595</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J25" t="inlineStr"/>
@@ -1855,7 +1859,7 @@
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
-          <t>571</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J26" t="inlineStr"/>
@@ -1903,7 +1907,7 @@
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>512</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J27" t="inlineStr"/>
@@ -1991,7 +1995,7 @@
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>456</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J29" t="inlineStr"/>
@@ -2039,7 +2043,7 @@
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
-          <t>605</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="J30" t="inlineStr"/>
@@ -2086,17 +2090,17 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>211 tests</t>
+          <t>355 tests</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>16544</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>211</t>
+          <t>355</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2159,7 +2163,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>7594</t>
+          <t>4000</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -2179,7 +2183,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>0</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -2667,7 +2671,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
     </row>
@@ -2679,7 +2683,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2695,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
     </row>
@@ -2715,7 +2719,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>PASS 1</t>
+          <t>PASS 2</t>
         </is>
       </c>
     </row>
@@ -2861,7 +2865,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>714</t>
+          <t>921</t>
         </is>
       </c>
     </row>
@@ -2898,7 +2902,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>89</t>
+          <t>161</t>
         </is>
       </c>
     </row>
@@ -2935,7 +2939,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>136</t>
+          <t>140</t>
         </is>
       </c>
     </row>
@@ -2968,7 +2972,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>211</t>
+          <t>355</t>
         </is>
       </c>
     </row>
@@ -3005,7 +3009,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>119</t>
+          <t>163</t>
         </is>
       </c>
     </row>
@@ -3064,7 +3068,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>architecture-drift.yml, docs.yml, eval-harness-ci.yml, merge-gate-audit.yml, merge-gate-seed.yml, merge-gate-verdict.yml, nightly-e2e.yml, outcome-labeller.yml, phoenix-live.yml, quality-gates.yml</t>
+          <t>architecture-drift.yml, docs.yml, eval-harness-ci.yml, merge-gate-audit.yml, merge-gate-seed.yml, merge-gate-verdict.yml, nightly-e2e.yml, outcome-labeller.yml, phoenix-live.yml, quality-gates.yml, required-check-stubs.yml, secret-scan.yml</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -3079,7 +3083,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>995</t>
+          <t>2571</t>
         </is>
       </c>
     </row>
@@ -3112,7 +3116,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>995</t>
+          <t>2571</t>
         </is>
       </c>
     </row>
@@ -3311,7 +3315,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>09337aec16e8b10588efd0e61c9d270d18ada1c4</t>
+          <t>0b2cbfb7c3f5b976bdcafcbd4ee8ff5c0959d632</t>
         </is>
       </c>
     </row>
@@ -3323,7 +3327,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>cursor/posix-e2e-driver-c319</t>
         </is>
       </c>
     </row>
@@ -3335,7 +3339,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-08-19T03:28:29+00:00</t>
+          <t>2026-09-06T21:29:05+00:00</t>
         </is>
       </c>
     </row>
@@ -3347,7 +3351,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Windows-10-10.0.26200-SP0</t>
+          <t>Linux-6.12.94+-x86_64-with-glibc2.39</t>
         </is>
       </c>
     </row>
@@ -3359,7 +3363,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>3.11.9</t>
+          <t>3.12.3</t>
         </is>
       </c>
     </row>
@@ -3371,7 +3375,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>pwsh -NoProfile -File scripts/run_all_e2e.ps1 -Tiers all -HypothesisProfile ci</t>
+          <t>bash scripts/run_all_e2e.sh --tiers all --hypothesis-profile ci</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(ci): POSIX e2e driver and CI-restored e2e-matrix freshness (#193)
scripts/run_all_e2e.sh mirrors the PowerShell driver (same tiers, step
inventory, report layout, anti-vacuous guards) so the nightly workflow
can produce a run report on ubuntu-latest; tests/test_e2e_driver_parity.py
fails if the two drivers drift. Freshness becomes CI-runnable via two
fixes: the Duration (ms) column is masked in the comparison (wall-clock
values can never reproduce across machines), and the committed artifact
is regenerated from the canonical Linux environment. nightly-e2e.yml
gains a single-version e2e-freshness job running driver + --check.

Co-authored-by: Cursor Agent <cursoragent@cursor.com>
Co-authored-by: Ian Cruickshank <ianshank@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/e2e-matrix/e2e-test-matrix.xlsx
+++ b/docs/e2e-matrix/e2e-test-matrix.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage Grid" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Credentials" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Provenance" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Test Matrix" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Coverage Grid" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Credentials" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Provenance" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Matrix'!$A$1:$N$41</definedName>
@@ -570,17 +570,17 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>714 tests</t>
+          <t>921 tests</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>47591</t>
+          <t>10000</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>714</t>
+          <t>921</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -638,17 +638,17 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>89 tests</t>
+          <t>161 tests</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>20250</t>
+          <t>23000</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>89</t>
+          <t>161</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -706,17 +706,17 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>136 tests</t>
+          <t>140 tests</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>6791</t>
+          <t>2000</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>136</t>
+          <t>140</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -774,17 +774,17 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>119 tests</t>
+          <t>163 tests</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>4876</t>
+          <t>2000</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>119</t>
+          <t>163</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2389</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -910,22 +910,22 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>995 tests</t>
+          <t>2571 tests</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>40601</t>
+          <t>56000</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>995</t>
+          <t>2571</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>28</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -978,22 +978,22 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>995 tests</t>
+          <t>2571 tests</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>39940</t>
+          <t>55000</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>995</t>
+          <t>2571</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>28</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1047,7 +1047,7 @@
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>33088</t>
+          <t>20000</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
@@ -1087,22 +1087,26 @@
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>NOT-RUN</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>not reached in this run</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>artifacts/e2e-report/matrix_coverage-check.log</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1139,7 +1143,7 @@
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>516</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
@@ -1187,7 +1191,7 @@
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>506</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
@@ -1235,7 +1239,7 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>531</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
@@ -1283,7 +1287,7 @@
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>1166</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
@@ -1371,7 +1375,7 @@
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>595</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
@@ -1419,7 +1423,7 @@
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
@@ -1467,7 +1471,7 @@
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>1094</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
@@ -1515,7 +1519,7 @@
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>1045</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
@@ -1563,7 +1567,7 @@
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>1114</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="J20" t="inlineStr"/>
@@ -1611,7 +1615,7 @@
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>1173</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J21" t="inlineStr"/>
@@ -1659,7 +1663,7 @@
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>1144</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
@@ -1707,7 +1711,7 @@
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>1098</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J23" t="inlineStr"/>
@@ -1754,12 +1758,12 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>decision exit 10</t>
+          <t>decision</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>534</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J24" t="inlineStr"/>
@@ -1807,7 +1811,7 @@
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>595</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J25" t="inlineStr"/>
@@ -1855,7 +1859,7 @@
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
-          <t>571</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J26" t="inlineStr"/>
@@ -1903,7 +1907,7 @@
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>512</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J27" t="inlineStr"/>
@@ -1991,7 +1995,7 @@
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>456</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J29" t="inlineStr"/>
@@ -2039,7 +2043,7 @@
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
-          <t>605</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="J30" t="inlineStr"/>
@@ -2086,17 +2090,17 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>211 tests</t>
+          <t>355 tests</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>16544</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>211</t>
+          <t>355</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2159,7 +2163,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>7594</t>
+          <t>4000</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -2179,7 +2183,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>0</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -2667,7 +2671,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
     </row>
@@ -2679,7 +2683,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2695,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
     </row>
@@ -2715,7 +2719,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>PASS 1</t>
+          <t>PASS 2</t>
         </is>
       </c>
     </row>
@@ -2861,7 +2865,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>714</t>
+          <t>921</t>
         </is>
       </c>
     </row>
@@ -2898,7 +2902,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>89</t>
+          <t>161</t>
         </is>
       </c>
     </row>
@@ -2935,7 +2939,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>136</t>
+          <t>140</t>
         </is>
       </c>
     </row>
@@ -2968,7 +2972,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>211</t>
+          <t>355</t>
         </is>
       </c>
     </row>
@@ -3005,7 +3009,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>119</t>
+          <t>163</t>
         </is>
       </c>
     </row>
@@ -3064,7 +3068,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>architecture-drift.yml, docs.yml, eval-harness-ci.yml, merge-gate-audit.yml, merge-gate-seed.yml, merge-gate-verdict.yml, nightly-e2e.yml, outcome-labeller.yml, phoenix-live.yml, quality-gates.yml</t>
+          <t>architecture-drift.yml, docs.yml, eval-harness-ci.yml, merge-gate-audit.yml, merge-gate-seed.yml, merge-gate-verdict.yml, nightly-e2e.yml, outcome-labeller.yml, phoenix-live.yml, quality-gates.yml, required-check-stubs.yml, secret-scan.yml</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -3079,7 +3083,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>995</t>
+          <t>2571</t>
         </is>
       </c>
     </row>
@@ -3112,7 +3116,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>995</t>
+          <t>2571</t>
         </is>
       </c>
     </row>
@@ -3311,7 +3315,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>09337aec16e8b10588efd0e61c9d270d18ada1c4</t>
+          <t>0b2cbfb7c3f5b976bdcafcbd4ee8ff5c0959d632</t>
         </is>
       </c>
     </row>
@@ -3323,7 +3327,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>cursor/posix-e2e-driver-c319</t>
         </is>
       </c>
     </row>
@@ -3335,7 +3339,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-08-19T03:28:29+00:00</t>
+          <t>2026-09-06T21:29:05+00:00</t>
         </is>
       </c>
     </row>
@@ -3347,7 +3351,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Windows-10-10.0.26200-SP0</t>
+          <t>Linux-6.12.94+-x86_64-with-glibc2.39</t>
         </is>
       </c>
     </row>
@@ -3359,7 +3363,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>3.11.9</t>
+          <t>3.12.3</t>
         </is>
       </c>
     </row>
@@ -3371,7 +3375,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>pwsh -NoProfile -File scripts/run_all_e2e.ps1 -Tiers all -HypothesisProfile ci</t>
+          <t>bash scripts/run_all_e2e.sh --tiers all --hypothesis-profile ci</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: restamp e2e-matrix from a 31/31 offline POSIX driver
Regenerate docs/e2e-matrix from run_all_e2e.sh --tiers offline (PASS 31 /
FAIL 0 / SKIP 0, suite:root 2978). Retire ERRATA provenance and monotonicity
waivers. Archive openspec/changes/repair-e2e-matrix-provenance.

Co-authored-by: Ian Cruickshank <ianshank@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/e2e-matrix/e2e-test-matrix.xlsx
+++ b/docs/e2e-matrix/e2e-test-matrix.xlsx
@@ -575,7 +575,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>35404</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -643,7 +643,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>23000</t>
+          <t>23540</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -711,7 +711,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2000</t>
+          <t>2052</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2000</t>
+          <t>7285</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>517</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -910,22 +910,22 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2571 tests</t>
+          <t>2978 tests</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>56000</t>
+          <t>70737</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2571</t>
+          <t>2978</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>32</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -978,22 +978,22 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2571 tests</t>
+          <t>2978 tests</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>55000</t>
+          <t>71836</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2571</t>
+          <t>2978</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>32</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1047,7 +1047,7 @@
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>20000</t>
+          <t>20417</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
@@ -1095,7 +1095,7 @@
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>631</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
@@ -1143,7 +1143,7 @@
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>56</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
@@ -1191,7 +1191,7 @@
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>86</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
@@ -1239,7 +1239,7 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>86</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
@@ -1287,7 +1287,7 @@
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>718</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
@@ -1375,7 +1375,7 @@
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>87</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
@@ -1423,7 +1423,7 @@
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>89</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
@@ -1471,7 +1471,7 @@
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>383</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
@@ -1519,7 +1519,7 @@
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>375</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
@@ -1567,7 +1567,7 @@
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>384</t>
         </is>
       </c>
       <c r="J20" t="inlineStr"/>
@@ -1615,7 +1615,7 @@
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>375</t>
         </is>
       </c>
       <c r="J21" t="inlineStr"/>
@@ -1663,7 +1663,7 @@
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>411</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
@@ -1711,7 +1711,7 @@
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>398</t>
         </is>
       </c>
       <c r="J23" t="inlineStr"/>
@@ -1758,12 +1758,12 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>decision</t>
+          <t>decision exit 10</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>86</t>
         </is>
       </c>
       <c r="J24" t="inlineStr"/>
@@ -1811,7 +1811,7 @@
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>97</t>
         </is>
       </c>
       <c r="J25" t="inlineStr"/>
@@ -1859,7 +1859,7 @@
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>86</t>
         </is>
       </c>
       <c r="J26" t="inlineStr"/>
@@ -1907,7 +1907,7 @@
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>90</t>
         </is>
       </c>
       <c r="J27" t="inlineStr"/>
@@ -1995,7 +1995,7 @@
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>51</t>
         </is>
       </c>
       <c r="J29" t="inlineStr"/>
@@ -2043,7 +2043,7 @@
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>107</t>
         </is>
       </c>
       <c r="J30" t="inlineStr"/>
@@ -2158,17 +2158,17 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>85 tests</t>
+          <t>92 tests</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>4000</t>
+          <t>4474</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>92</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -3068,7 +3068,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>architecture-drift.yml, docs.yml, eval-harness-ci.yml, merge-gate-audit.yml, merge-gate-seed.yml, merge-gate-verdict.yml, nightly-e2e.yml, outcome-labeller.yml, phoenix-live.yml, quality-gates.yml, required-check-stubs.yml, secret-scan.yml</t>
+          <t>architecture-drift.yml, docs.yml, eval-harness-ci.yml, merge-gate-audit.yml, merge-gate-seed.yml, merge-gate-verdict.yml, nightly-e2e.yml, outcome-labeller.yml, phoenix-live.yml, pip-audit.yml, quality-gates.yml, required-check-stubs.yml, secret-scan.yml</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2571</t>
+          <t>2978</t>
         </is>
       </c>
     </row>
@@ -3116,7 +3116,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2571</t>
+          <t>2978</t>
         </is>
       </c>
     </row>
@@ -3315,7 +3315,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0b2cbfb7c3f5b976bdcafcbd4ee8ff5c0959d632</t>
+          <t>27e5b8cb588569f021e8bc83b7592fa67be91015</t>
         </is>
       </c>
     </row>
@@ -3327,7 +3327,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>cursor/posix-e2e-driver-c319</t>
+          <t>cursor/e2e-matrix-restamp-24d8</t>
         </is>
       </c>
     </row>
@@ -3339,7 +3339,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-06T21:29:05+00:00</t>
+          <t>2026-09-09T01:57:55+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>